<commit_message>
feat(funnel): retire ecolabel workshop + wire in-Excel upsell to ESG Passport
Funnel is now tool -> free baseline -> ESG Passport.

Workshop (discontinued) removed everywhere: ecolabel tool CTA, ArticleCTA
footnote/link, products page card, Footer, for-advisors, SiteSearch + search
index; workshop page deleted and redirected to /tools/ecolabel-selector.
Dropped "workshop" from the SearchEntry type union for Record consistency.

In-Excel upsell: both authored workbooks (biofuels, ecolabel) now carry a
"Your next steps" band + notes ladder — free baseline (ecosystemsunited.com/
tracker) then ESG Passport (EUR 499 one-time, LemonSqueezy checkout).
Framed honestly as "answer the ESG/Scope-3 questionnaires your buyers send"
because Passport is not GlobalG.A.P./farm-capable yet.

Verified: clean production build (exit 0), workshop route gone, all four
tool routes present.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/biofuel-feedstock-sustainability-comparison.xlsx
+++ b/public/downloads/biofuel-feedstock-sustainability-comparison.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
   <si>
     <t>Biofuel Feedstock Sustainability Comparison</t>
   </si>
@@ -88,6 +88,15 @@
     <t>Scores are directional (1 = poor, 5 = strong), synthesised from published biofuel-generation research for orientation — not a lab-grade lifecycle assessment. See Notes &amp; Sources.</t>
   </si>
   <si>
+    <t>Ready to act on this? Your next steps</t>
+  </si>
+  <si>
+    <t>1)  Build your free operational baseline  →  ecosystemsunited.com/tracker</t>
+  </si>
+  <si>
+    <t>2)  Answer the ESG &amp; Scope-3 questionnaires your buyers send, straight from your data  →  ESG Passport · €499 one-time, yours to own, no subscription</t>
+  </si>
+  <si>
     <t>Score It For Your Operation</t>
   </si>
   <si>
@@ -157,7 +166,13 @@
     <t>Use it, then go further</t>
   </si>
   <si>
-    <t xml:space="preserve">  Pair this with the interactive tool at ecosystemsunited.com/tools/biofuel-feedstock-compare, and build the operational baseline that lets you evaluate your own waste streams: ecosystemsunited.com/tracker (free).</t>
+    <t xml:space="preserve">  1) Pair this with the interactive tool at ecosystemsunited.com/tools/biofuel-feedstock-compare.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  2) Build the free operational baseline that lets you evaluate your own waste streams: ecosystemsunited.com/tracker.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3) When buyers send ESG or Scope-3 questionnaires, answer them from your data with ESG Passport — €499 one-time, yours to own, no subscription.</t>
   </si>
   <si>
     <t>© Ecosystems United — Five Stacks Framework. Free to share.</t>
@@ -167,7 +182,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -203,14 +218,25 @@
       <sz val="9"/>
     </font>
     <font>
-      <color rgb="FF999999"/>
-    </font>
-    <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
+      <u/>
+      <color rgb="FF3D2E7C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <color rgb="FF1B6F55"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="FF999999"/>
+    </font>
+    <font>
       <i/>
       <color rgb="FF666666"/>
       <sz val="9"/>
@@ -224,7 +250,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -263,6 +289,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFEAF6F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF7D6"/>
       </patternFill>
     </fill>
@@ -294,7 +325,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -332,29 +363,38 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="9" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -696,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -866,12 +906,46 @@
       <c r="D13" s="12"/>
       <c r="E13" s="12"/>
     </row>
+    <row r="15" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+    </row>
+    <row r="17" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A17:E17"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A16" r:id="rId1"/>
+    <hyperlink ref="A17" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -889,7 +963,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -899,7 +973,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -908,42 +982,42 @@
       <c r="F2" s="2"/>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="16" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="17">
         <v>1</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="18">
         <v>2</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="18">
         <v>4</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="18">
         <v>5</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="18">
         <v>5</v>
       </c>
     </row>
@@ -951,19 +1025,19 @@
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="17">
         <v>1</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="18">
         <v>2</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="18">
         <v>4</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="18">
         <v>4</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="18">
         <v>5</v>
       </c>
     </row>
@@ -971,19 +1045,19 @@
       <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="17">
         <v>1</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="18">
         <v>1</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="18">
         <v>4</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="18">
         <v>5</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="18">
         <v>5</v>
       </c>
     </row>
@@ -991,19 +1065,19 @@
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="17">
         <v>1</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="18">
         <v>3</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="18">
         <v>4</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="18">
         <v>2</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="18">
         <v>3</v>
       </c>
     </row>
@@ -1011,51 +1085,51 @@
       <c r="A9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="17">
         <v>1</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="18">
         <v>5</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="18">
         <v>3</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="18">
         <v>2</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="18">
+      <c r="A10" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="21">
         <f>IF(SUM($B$5:$B$9)=0,0,SUMPRODUCT($B$5:$B$9,C5:C9)/(SUM($B$5:$B$9)*5))</f>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="21">
         <f>IF(SUM($B$5:$B$9)=0,0,SUMPRODUCT($B$5:$B$9,D5:D9)/(SUM($B$5:$B$9)*5))</f>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="21">
         <f>IF(SUM($B$5:$B$9)=0,0,SUMPRODUCT($B$5:$B$9,E5:E9)/(SUM($B$5:$B$9)*5))</f>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="21">
         <f>IF(SUM($B$5:$B$9)=0,0,SUMPRODUCT($B$5:$B$9,F5:F9)/(SUM($B$5:$B$9)*5))</f>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="A12" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1076,7 +1150,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -1084,102 +1158,112 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="23" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
-        <v>31</v>
-      </c>
-    </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
-        <v>35</v>
+      <c r="A5" s="24" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
-        <v>36</v>
+      <c r="A6" s="23" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="20" t="s">
-        <v>37</v>
+      <c r="A7" s="23" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="20" t="s">
-        <v>38</v>
+      <c r="A8" s="23" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
-        <v>39</v>
+      <c r="A9" s="23" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
-        <v>40</v>
+      <c r="A10" s="23" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
-        <v>31</v>
+      <c r="A11" s="23" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
-        <v>41</v>
+      <c r="A12" s="24" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="13" ht="66" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="20" t="s">
-        <v>42</v>
+      <c r="A13" s="23" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="20" t="s">
-        <v>31</v>
+      <c r="A14" s="23" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
-        <v>43</v>
+      <c r="A15" s="24" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="16" ht="66" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
-        <v>44</v>
+      <c r="A16" s="23" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="20" t="s">
-        <v>31</v>
+      <c r="A17" s="23" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="19" ht="51" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="20" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="20" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="20" t="s">
-        <v>47</v>
+      <c r="A18" s="24" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="23" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="23" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="23" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>